<commit_message>
Update konten artikel tanggal 31 agustus 2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98CD6915-A2A7-43B2-83A5-97AF88759A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74BC6DB-4876-4320-9C54-814A68582D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2015,18 +2015,18 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2037,10 +2037,10 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2354,20 +2354,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2378,65 +2378,65 @@
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
     </row>
     <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
@@ -2600,55 +2600,55 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="39"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="34" t="s">
+      <c r="B25" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="39"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B26" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="39"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
@@ -2694,15 +2694,15 @@
       <c r="A1" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
     </row>
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -3082,16 +3082,16 @@
       <c r="A1" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="2" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -4208,16 +4208,16 @@
       <c r="A1" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="2" spans="1:11" ht="56.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="11" t="s">
@@ -4255,108 +4255,108 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="I3" s="19" t="s">
-        <v>115</v>
+      <c r="C3" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>136</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>169</v>
+        <v>191</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>173</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>106</v>
+      <c r="C4" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>136</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="K4" s="16" t="s">
-        <v>177</v>
+        <v>199</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B5" s="18" t="s">
+      <c r="A5" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>66</v>
+      <c r="C5" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>136</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>184</v>
+        <v>207</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -4385,12 +4385,12 @@
       <c r="A1" s="43" t="s">
         <v>386</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -4577,12 +4577,12 @@
       <c r="A1" s="43" t="s">
         <v>425</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -4814,9 +4814,9 @@
       <c r="A1" s="43" t="s">
         <v>462</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="3" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
@@ -4917,52 +4917,52 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="41" t="s">
         <v>490</v>
       </c>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
     </row>
     <row r="12" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="45" t="s">
         <v>491</v>
       </c>
-      <c r="B12" s="36"/>
+      <c r="B12" s="39"/>
       <c r="C12" s="44" t="s">
         <v>492</v>
       </c>
-      <c r="D12" s="36"/>
+      <c r="D12" s="39"/>
     </row>
     <row r="13" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="45" t="s">
         <v>493</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="39"/>
       <c r="C13" s="44" t="s">
         <v>494</v>
       </c>
-      <c r="D13" s="36"/>
+      <c r="D13" s="39"/>
     </row>
     <row r="14" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="45" t="s">
         <v>495</v>
       </c>
-      <c r="B14" s="36"/>
+      <c r="B14" s="39"/>
       <c r="C14" s="44" t="s">
         <v>496</v>
       </c>
-      <c r="D14" s="36"/>
+      <c r="D14" s="39"/>
     </row>
     <row r="15" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="45" t="s">
         <v>497</v>
       </c>
-      <c r="B15" s="36"/>
+      <c r="B15" s="39"/>
       <c r="C15" s="44" t="s">
         <v>498</v>
       </c>
-      <c r="D15" s="36"/>
+      <c r="D15" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -4999,20 +4999,20 @@
       <c r="A1" s="43" t="s">
         <v>499</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="47" t="s">
         <v>500</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
     </row>
     <row r="4" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
@@ -5021,12 +5021,12 @@
       <c r="B4" s="3" t="s">
         <v>502</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="37" t="s">
         <v>503</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
       <c r="G4" s="25" t="s">
         <v>504</v>
       </c>
@@ -5038,12 +5038,12 @@
       <c r="B5" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="37" t="s">
         <v>507</v>
       </c>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="39"/>
       <c r="G5" s="25" t="s">
         <v>504</v>
       </c>
@@ -5055,12 +5055,12 @@
       <c r="B6" s="3" t="s">
         <v>509</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="37" t="s">
         <v>510</v>
       </c>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="25" t="s">
         <v>511</v>
       </c>
@@ -5072,12 +5072,12 @@
       <c r="B7" s="3" t="s">
         <v>513</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="37" t="s">
         <v>514</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="36"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="25" t="s">
         <v>504</v>
       </c>
@@ -5089,12 +5089,12 @@
       <c r="B8" s="3" t="s">
         <v>516</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="37" t="s">
         <v>517</v>
       </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="36"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="39"/>
       <c r="G8" s="25" t="s">
         <v>504</v>
       </c>
@@ -5106,26 +5106,26 @@
       <c r="B9" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="37" t="s">
         <v>520</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="39"/>
       <c r="G9" s="25" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="46" t="s">
         <v>521</v>
       </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
     </row>
     <row r="13" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
@@ -5221,15 +5221,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5253,12 +5253,12 @@
       <c r="A1" s="43" t="s">
         <v>542</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">

</xml_diff>

<commit_message>
Update artikel tanggal 1 september 2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74BC6DB-4876-4320-9C54-814A68582D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B327DF-7F3C-42C8-9ABF-E26EEA851E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2037,10 +2037,10 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4255,108 +4255,108 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B3" s="20" t="s">
+      <c r="A3" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>189</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="I3" s="21" t="s">
-        <v>136</v>
+      <c r="C3" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>129</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>192</v>
+        <v>215</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B4" s="18" t="s">
+      <c r="A4" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>136</v>
+      <c r="C4" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>218</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>129</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>200</v>
+        <v>223</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>201</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>202</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>205</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>136</v>
+      <c r="C5" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>129</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="K5" s="16" t="s">
-        <v>208</v>
+        <v>230</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -5007,7 +5007,7 @@
       <c r="G1" s="35"/>
     </row>
     <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="46" t="s">
         <v>500</v>
       </c>
       <c r="B3" s="35"/>
@@ -5117,7 +5117,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="46" t="s">
+      <c r="A12" s="47" t="s">
         <v>521</v>
       </c>
       <c r="B12" s="35"/>

</xml_diff>

<commit_message>
update artikel tanggal 2 sep2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B327DF-7F3C-42C8-9ABF-E26EEA851E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C56E83-A7C9-4DE7-96C6-9F4970966A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4255,108 +4255,108 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>212</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>214</v>
-      </c>
-      <c r="I3" s="19" t="s">
-        <v>129</v>
+      <c r="C3" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>115</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>216</v>
+        <v>238</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
-        <v>209</v>
-      </c>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>217</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>219</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>221</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>222</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>129</v>
+      <c r="C4" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>143</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="K4" s="16" t="s">
-        <v>224</v>
+        <v>245</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B5" s="18" t="s">
+      <c r="A5" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>225</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>129</v>
+      <c r="C5" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>143</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>231</v>
+        <v>252</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update artikel tanggal 2 sep 2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C56E83-A7C9-4DE7-96C6-9F4970966A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87E80E3-6D06-48AE-B3F5-AFA627F6D321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4255,108 +4255,108 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>232</v>
-      </c>
-      <c r="B3" s="20" t="s">
+      <c r="A3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>234</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>235</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>236</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>237</v>
-      </c>
-      <c r="I3" s="21" t="s">
-        <v>115</v>
+      <c r="C3" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>136</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>239</v>
+        <v>260</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="B4" s="18" t="s">
+      <c r="A4" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>241</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>143</v>
+      <c r="C4" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>136</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>246</v>
+        <v>267</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
-        <v>232</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>247</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>248</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>249</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>250</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>251</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>143</v>
+      <c r="C5" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>136</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="K5" s="16" t="s">
-        <v>253</v>
+        <v>274</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update artikel tanggal 4 sep 2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87E80E3-6D06-48AE-B3F5-AFA627F6D321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DE7CA4-A159-42F3-89CD-8F36CCE8B12E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4255,108 +4255,108 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="I3" s="19" t="s">
-        <v>136</v>
+      <c r="C3" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>106</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>261</v>
+        <v>282</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
-        <v>254</v>
-      </c>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>262</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>263</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>264</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>265</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>266</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>136</v>
+      <c r="C4" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>66</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="K4" s="16" t="s">
-        <v>268</v>
+        <v>289</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="B5" s="18" t="s">
+      <c r="A5" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>270</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>136</v>
+      <c r="C5" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>292</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>96</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>275</v>
+        <v>296</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update artikel 9 sep 2026
</commit_message>
<xml_diff>
--- a/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
+++ b/strategi-seo-aeo-geo-vendoroutbound-v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GM ACADEMY\PROJECT VENDOR OUTBOUND ID\PROJECT YANG SUDAH DIDEPLOY DOMAIN\venroroutboundid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DE7CA4-A159-42F3-89CD-8F36CCE8B12E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E86FEB5-0569-4758-B30A-7AE1825904CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1924,7 +1924,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2041,6 +2041,34 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4254,109 +4282,109 @@
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="B3" s="20" t="s">
+    <row r="3" spans="1:11" s="48" customFormat="1" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="49" t="s">
+        <v>342</v>
+      </c>
+      <c r="B3" s="54" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>279</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>280</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>281</v>
-      </c>
-      <c r="I3" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="B4" s="18" t="s">
+      <c r="C3" s="51" t="s">
+        <v>343</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>344</v>
+      </c>
+      <c r="E3" s="55" t="s">
+        <v>144</v>
+      </c>
+      <c r="F3" s="51" t="s">
+        <v>345</v>
+      </c>
+      <c r="G3" s="51" t="s">
+        <v>346</v>
+      </c>
+      <c r="H3" s="51" t="s">
+        <v>347</v>
+      </c>
+      <c r="I3" s="55" t="s">
+        <v>143</v>
+      </c>
+      <c r="J3" s="50" t="s">
+        <v>348</v>
+      </c>
+      <c r="K3" s="51" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="48" customFormat="1" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="B4" s="56" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>284</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>286</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>287</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>288</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="C4" s="53" t="s">
+        <v>350</v>
+      </c>
+      <c r="D4" s="57" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4" s="57" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="53" t="s">
+        <v>352</v>
+      </c>
+      <c r="G4" s="53" t="s">
+        <v>353</v>
+      </c>
+      <c r="H4" s="53" t="s">
+        <v>354</v>
+      </c>
+      <c r="I4" s="57" t="s">
+        <v>143</v>
+      </c>
+      <c r="J4" s="50" t="s">
+        <v>355</v>
+      </c>
+      <c r="K4" s="53" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="48" customFormat="1" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="49" t="s">
+        <v>342</v>
+      </c>
+      <c r="B5" s="54" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>292</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>293</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>294</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>295</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="K5" s="16" t="s">
-        <v>297</v>
+      <c r="C5" s="51" t="s">
+        <v>357</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>358</v>
+      </c>
+      <c r="E5" s="55" t="s">
+        <v>144</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>359</v>
+      </c>
+      <c r="G5" s="51" t="s">
+        <v>360</v>
+      </c>
+      <c r="H5" s="51" t="s">
+        <v>361</v>
+      </c>
+      <c r="I5" s="55" t="s">
+        <v>143</v>
+      </c>
+      <c r="J5" s="50" t="s">
+        <v>362</v>
+      </c>
+      <c r="K5" s="51" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>